<commit_message>
📊 Horarios actualizados Línea 141 - 2367
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:43:24</t>
+          <t>Última actualización: 02:16:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>00:43:24</t>
+          <t>02:16:16</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:12</t>
+          <t>02:58</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,12 +498,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>00:43:24</t>
+          <t>02:16:16</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>01:58</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -512,9 +512,34 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>02:16:16</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>04:01</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>105</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -544,7 +569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:43:24</t>
+          <t>Última actualización: 02:16:16</t>
         </is>
       </c>
     </row>
@@ -585,12 +610,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>00:43:24</t>
+          <t>02:16:16</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:12</t>
+          <t>02:58</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -599,7 +624,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -631,7 +656,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:43:24</t>
+          <t>Última actualización: 02:16:16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2368
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:16:16</t>
+          <t>Última actualización: 03:14:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:16:16</t>
+          <t>03:14:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>02:58</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:16:16</t>
+          <t>03:14:40</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,23 +523,48 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:16:16</t>
+          <t>03:14:40</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:01</t>
+          <t>04:45</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>03:14:40</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:53</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>99</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -569,7 +594,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:16:16</t>
+          <t>Última actualización: 03:14:40</t>
         </is>
       </c>
     </row>
@@ -610,21 +635,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:16:16</t>
+          <t>03:14:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>02:58</t>
+          <t>04:45</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>42</v>
+        <v>91</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -656,7 +681,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:16:16</t>
+          <t>Última actualización: 03:14:40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2369
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:14:40</t>
+          <t>Última actualización: 04:17:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:14:40</t>
+          <t>04:17:33</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:46</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03:14:40</t>
+          <t>04:17:33</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:01</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03:14:40</t>
+          <t>04:17:33</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:45</t>
+          <t>05:16</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>91</v>
+        <v>59</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,23 +548,173 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03:14:40</t>
+          <t>04:17:33</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>99</v>
+        <v>65</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>04:17:33</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>05:34</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>77</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>04:17:33</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>05:46</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>89</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>04:17:33</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>05:54</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>97</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>04:17:33</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06:04</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>107</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>04:17:33</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>114</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>04:17:33</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06:14</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>117</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -581,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -594,14 +744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:14:40</t>
+          <t>Última actualización: 04:17:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -635,12 +785,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:14:40</t>
+          <t>04:17:33</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:45</t>
+          <t>04:46</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -649,9 +799,59 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>91</v>
+        <v>29</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>04:17:33</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>05:34</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>77</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>04:17:33</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>114</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -668,7 +868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -681,14 +881,91 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:14:40</t>
+          <t>Última actualización: 04:17:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>04:17:33</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>05:44</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>87</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>04:17:33</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>115</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2370
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:17:33</t>
+          <t>Última actualización: 04:58:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:17:33</t>
+          <t>04:58:08</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:17</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>65</v>
+        <v>19</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:17:33</t>
+          <t>04:58:08</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:34</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>77</v>
+        <v>24</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -603,16 +603,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:46</t>
+          <t>05:34</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:17:33</t>
+          <t>04:58:08</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>05:54</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>97</v>
+        <v>46</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -653,16 +653,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:04</t>
+          <t>05:46</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:17:33</t>
+          <t>04:58:08</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:11</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>114</v>
+        <v>49</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -703,18 +703,293 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>05:54</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>97</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>04:58:08</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>63</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>04:17:33</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06:04</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>107</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>04:58:08</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>06:09</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>71</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>04:17:33</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>114</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>04:58:08</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>74</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>04:17:33</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>06:14</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>225_C ROCA-H SUR</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D21" t="n">
         <v>117</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>04:58:08</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>92</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>04:58:08</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>06:36</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>98</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>04:58:08</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>101</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>04:58:08</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>103</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>04:58:08</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>103</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -731,7 +1006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -744,14 +1019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:17:33</t>
+          <t>Última actualización: 04:58:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -852,6 +1127,31 @@
         <v>114</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>04:58:08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>74</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -881,7 +1181,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:17:33</t>
+          <t>Última actualización: 04:58:08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2371
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:58:08</t>
+          <t>Última actualización: 05:38:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:58:08</t>
+          <t>05:38:37</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>46</v>
+        <v>6</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:58:08</t>
+          <t>05:38:37</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>49</v>
+        <v>9</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>04:58:08</t>
+          <t>05:38:37</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>71</v>
+        <v>31</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>04:58:08</t>
+          <t>05:38:37</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -837,7 +837,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>04:58:08</t>
+          <t>05:38:37</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>92</v>
+        <v>52</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>04:58:08</t>
+          <t>05:38:37</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>04:58:08</t>
+          <t>05:38:37</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>101</v>
+        <v>61</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>04:58:08</t>
+          <t>05:38:37</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,13 +983,213 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>63</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>05:38:37</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>06:59</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>81</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>05:38:37</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>84</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>05:38:37</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>07:10</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="D29" t="n">
+        <v>92</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>05:38:37</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
         <v>103</v>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>05:38:37</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>07:26</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>108</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>05:38:37</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>07:27</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>109</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>05:38:37</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>113</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>05:38:37</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>118</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1006,7 +1206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1019,14 +1219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:58:08</t>
+          <t>Última actualización: 05:38:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1335,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:58:08</t>
+          <t>05:38:37</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1149,9 +1349,59 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>05:38:37</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>84</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>05:38:37</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>113</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1181,7 +1431,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:58:08</t>
+          <t>Última actualización: 05:38:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2372
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:38:37</t>
+          <t>Última actualización: 06:23:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>05:38:37</t>
+          <t>06:23:26</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>52</v>
+        <v>7</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>05:38:37</t>
+          <t>06:23:26</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>58</v>
+        <v>13</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>05:38:37</t>
+          <t>06:23:26</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>61</v>
+        <v>16</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,7 +948,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>04:58:08</t>
+          <t>06:23:26</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>103</v>
+        <v>18</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>05:38:37</t>
+          <t>06:23:26</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>05:38:37</t>
+          <t>06:23:26</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>81</v>
+        <v>36</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>05:38:37</t>
+          <t>06:23:26</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>84</v>
+        <v>39</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>05:38:37</t>
+          <t>06:23:26</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:16</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>05:38:37</t>
+          <t>06:23:26</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>108</v>
+        <v>58</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,21 +1123,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>05:38:37</t>
+          <t>06:23:26</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>109</v>
+        <v>63</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,21 +1148,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>05:38:37</t>
+          <t>06:23:26</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>113</v>
+        <v>64</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,23 +1173,123 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>05:38:37</t>
+          <t>06:23:26</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>68</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>06:23:26</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>07:36</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>118</v>
-      </c>
-      <c r="E34" t="inlineStr">
+      <c r="D35" t="n">
+        <v>73</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>06:23:26</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>81</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>06:23:26</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>88</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>06:23:26</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>116</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1206,7 +1306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1219,14 +1319,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:38:37</t>
+          <t>Última actualización: 06:23:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1460,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:38:37</t>
+          <t>06:23:26</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1374,7 +1474,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>84</v>
+        <v>39</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1385,7 +1485,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:38:37</t>
+          <t>06:23:26</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1399,9 +1499,34 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>113</v>
+        <v>68</v>
       </c>
       <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>06:23:26</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>88</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1418,7 +1543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1431,14 +1556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:38:37</t>
+          <t>Última actualización: 06:23:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -1514,6 +1639,31 @@
         <v>115</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:23:26</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>86</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2373
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:23:26</t>
+          <t>Última actualización: 07:01:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 44</t>
         </is>
       </c>
     </row>
@@ -1048,21 +1048,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>05:38:37</t>
+          <t>07:01:04</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>07:10</t>
+          <t>07:03</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>92</v>
+        <v>2</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>06:23:26</t>
+          <t>05:38:37</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>07:16</t>
+          <t>07:10</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>53</v>
+        <v>92</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1103,16 +1103,16 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:16</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,21 +1123,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06:23:26</t>
+          <t>07:01:04</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>63</v>
+        <v>20</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1153,16 +1153,16 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:23:26</t>
+          <t>07:01:04</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:23:26</t>
+          <t>07:01:04</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1228,16 +1228,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,21 +1248,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:23:26</t>
+          <t>07:01:04</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>07:51</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>88</v>
+        <v>31</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1278,18 +1278,293 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>73</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>07:01:04</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>36</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>07:01:04</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>43</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>06:23:26</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>88</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>07:01:04</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>07:52</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>51</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>07:01:04</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>08:06</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>65</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>07:01:04</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>08:19</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D38" t="n">
-        <v>116</v>
-      </c>
-      <c r="E38" t="inlineStr">
+      <c r="D44" t="n">
+        <v>78</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>07:01:04</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>08:22</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>81</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>07:01:04</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>08:26</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>85</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>07:01:04</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>100</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>07:01:04</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>104</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>07:01:04</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>104</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1306,7 +1581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1319,14 +1594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:23:26</t>
+          <t>Última actualización: 07:01:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -1485,21 +1760,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>06:23:26</t>
+          <t>07:01:04</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:03</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1515,18 +1790,143 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>68</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>07:01:04</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>31</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>06:23:26</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>07:51</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D14" t="n">
         <v>88</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>07:01:04</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>07:52</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>51</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>07:01:04</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>104</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>07:01:04</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>104</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1543,7 +1943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1556,14 +1956,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:23:26</t>
+          <t>Última actualización: 07:01:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -1664,6 +2064,56 @@
         <v>86</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:01:04</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:20</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>79</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07:01:04</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>97</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2374
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:01:04</t>
+          <t>Última actualización: 07:50:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 44</t>
+          <t>Total filas: 57</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>06:23:26</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>88</v>
+        <v>1</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,12 +1373,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:01:04</t>
+          <t>06:23:26</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>07:52</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>51</v>
+        <v>88</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:01:04</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>08:06</t>
+          <t>07:52</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>65</v>
+        <v>2</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:01:04</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>78</v>
+        <v>5</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:01:04</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>81</v>
+        <v>11</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>07:01:04</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>08:26</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>85</v>
+        <v>16</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>07:01:04</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:15</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1528,16 +1528,16 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>104</v>
+        <v>78</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,23 +1548,348 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>08:22</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>32</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>08:26</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>36</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>07:01:04</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>100</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
         <is>
           <t>08:45</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>55</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D49" t="n">
+      <c r="D53" t="n">
+        <v>55</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>74</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>77</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>09:12</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>82</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>87</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>87</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>94</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
         <v>104</v>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>105</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>09:38</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>108</v>
+      </c>
+      <c r="E62" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1581,7 +1906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1594,14 +1919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:01:04</t>
+          <t>Última actualización: 07:50:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -1860,7 +2185,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07:01:04</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1874,7 +2199,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1885,7 +2210,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>07:01:04</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1899,7 +2224,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>104</v>
+        <v>55</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1910,7 +2235,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>07:01:04</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1924,9 +2249,34 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>104</v>
+        <v>55</v>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>77</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1943,7 +2293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1956,14 +2306,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:01:04</t>
+          <t>Última actualización: 07:50:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -2097,25 +2447,100 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>31</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>07:01:04</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>08:38</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D11" t="n">
         <v>97</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>70</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>73</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2375
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:50:06</t>
+          <t>Última actualización: 08:17:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 57</t>
+          <t>Total filas: 71</t>
         </is>
       </c>
     </row>
@@ -1523,21 +1523,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>07:01:04</t>
+          <t>08:17:37</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>08:17</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>07:01:04</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>32</v>
+        <v>78</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:17:37</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>08:26</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>07:01:04</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:22</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>100</v>
+        <v>32</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:17:37</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:25</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>55</v>
+        <v>8</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1653,16 +1653,16 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:26</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>07:01:04</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>74</v>
+        <v>100</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,21 +1698,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:17:37</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>09:07</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:17:37</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>09:12</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>82</v>
+        <v>27</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1753,16 +1753,16 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>87</v>
+        <v>55</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1778,16 +1778,16 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>87</v>
+        <v>55</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:17:37</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>08:57</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>94</v>
+        <v>40</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:17:37</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>104</v>
+        <v>47</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,21 +1848,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:17:37</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>105</v>
+        <v>49</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1878,18 +1878,368 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>77</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>08:17:37</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>54</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>09:12</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>82</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>08:17:37</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>59</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>87</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>87</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>08:17:37</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>67</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>08:17:37</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>77</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>08:17:37</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>78</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
           <t>09:38</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C71" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D62" t="n">
+      <c r="D71" t="n">
         <v>108</v>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>08:17:37</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>09:49</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>92</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>08:17:37</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>09:49</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>92</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>08:17:37</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>94</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>08:17:37</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>99</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>08:17:37</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>107</v>
+      </c>
+      <c r="E76" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1906,7 +2256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1919,14 +2269,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:50:06</t>
+          <t>Última actualización: 08:17:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -2210,12 +2560,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:17:37</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2224,7 +2574,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2235,12 +2585,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:17:37</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2249,7 +2599,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2265,18 +2615,118 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>55</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>55</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>08:17:37</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>49</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>09:07</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="D21" t="n">
         <v>77</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>08:17:37</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>99</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2293,7 +2743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2306,14 +2756,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:50:06</t>
+          <t>Última actualización: 08:17:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -2447,7 +2897,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:17:37</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2461,7 +2911,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2497,12 +2947,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:17:37</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:57</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2511,7 +2961,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2527,18 +2977,68 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>70</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:17:37</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>09:02</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>45</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>09:03</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D15" t="n">
         <v>73</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2376
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:17:37</t>
+          <t>Última actualización: 08:46:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 71</t>
+          <t>Total filas: 82</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:17:37</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>08:57</t>
+          <t>08:46</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:17:37</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>08:53</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>47</v>
+        <v>7</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1853,16 +1853,16 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:57</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,21 +1873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>09:07</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:17:37</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1928,16 +1928,16 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>09:12</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:17:37</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1978,16 +1978,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,12 +1998,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>87</v>
+        <v>30</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:17:37</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>67</v>
+        <v>30</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,21 +2048,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:17:37</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:17:37</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>09:38</t>
+          <t>09:24</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>108</v>
+        <v>38</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>08:17:37</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>09:49</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>92</v>
+        <v>48</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,21 +2148,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:17:37</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>09:49</t>
+          <t>09:35</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>92</v>
+        <v>49</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:17:37</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>09:51</t>
+          <t>09:38</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:17:37</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>99</v>
+        <v>58</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2228,18 +2228,293 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
+          <t>09:49</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>92</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>08:17:37</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>09:49</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>92</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>65</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>09:52</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>66</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>69</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>08:17:37</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>99</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>75</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
           <t>10:04</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D76" t="n">
-        <v>107</v>
-      </c>
-      <c r="E76" t="inlineStr">
+      <c r="D83" t="n">
+        <v>78</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>89</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>98</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>108</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>118</v>
+      </c>
+      <c r="E87" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2256,7 +2531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2269,14 +2544,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:17:37</t>
+          <t>Última actualización: 08:46:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -2570,7 +2845,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -2595,7 +2870,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -2660,21 +2935,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>08:17:37</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:46</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2685,12 +2960,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>09:07</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2699,7 +2974,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>77</v>
+        <v>20</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -2710,23 +2985,73 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>07:50:06</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>77</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>69</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>08:17:37</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>09:56</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="D24" t="n">
         <v>99</v>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2743,7 +3068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2756,14 +3081,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:17:37</t>
+          <t>Última actualización: 08:46:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -2972,7 +3297,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2986,7 +3311,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>70</v>
+        <v>14</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -3022,7 +3347,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3036,11 +3361,86 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>73</v>
+        <v>17</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>42</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>92</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>104</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2377
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E87"/>
+  <dimension ref="A1:E98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:46:31</t>
+          <t>Última actualización: 09:01:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 82</t>
+          <t>Total filas: 93</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>06:23:26</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1</v>
+        <v>88</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:23:26</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>88</v>
+        <v>1</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1873,21 +1873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>09:03</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>09:03</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,21 +1923,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>09:07</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1978,16 +1978,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>09:12</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>30</v>
+        <v>82</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,12 +2048,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>87</v>
+        <v>15</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,12 +2073,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>87</v>
+        <v>15</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>38</v>
+        <v>87</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>48</v>
+        <v>87</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,21 +2148,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:23</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>09:38</t>
+          <t>09:24</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>108</v>
+        <v>38</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>08:17:37</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>09:49</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>92</v>
+        <v>33</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:17:37</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>09:49</t>
+          <t>09:35</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>92</v>
+        <v>49</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,21 +2273,21 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>09:51</t>
+          <t>09:38</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>09:52</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>66</v>
+        <v>41</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>69</v>
+        <v>43</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2353,16 +2353,16 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:49</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,21 +2373,21 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>08:17:37</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>09:49</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2403,16 +2403,16 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>09:51</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2428,16 +2428,16 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>09:52</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>09:53</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>98</v>
+        <v>52</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>108</v>
+        <v>53</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2503,18 +2503,293 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>69</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>08:17:37</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>99</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>09:01:57</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>60</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>09:01:57</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>10:03</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>62</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>78</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>89</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>09:01:57</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>83</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>09:01:57</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>93</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>09:01:57</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>102</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
           <t>10:44</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C96" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D87" t="n">
+      <c r="D96" t="n">
         <v>118</v>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>09:01:57</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>10:54</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>113</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>09:01:57</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>115</v>
+      </c>
+      <c r="E98" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2531,7 +2806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2544,14 +2819,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:46:31</t>
+          <t>Última actualización: 09:01:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -2845,7 +3120,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -2870,7 +3145,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -2895,7 +3170,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -2920,7 +3195,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -2960,7 +3235,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2974,7 +3249,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3010,12 +3285,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3024,7 +3299,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -3035,23 +3310,48 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>69</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>08:17:37</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>09:56</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D25" t="n">
         <v>99</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3068,7 +3368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3081,14 +3381,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:46:31</t>
+          <t>Última actualización: 09:01:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3372,12 +3672,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>09:28</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3386,7 +3686,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3402,43 +3702,168 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10:18</t>
+          <t>09:28</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>92</v>
+        <v>42</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>09:01:57</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>74</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>09:01:57</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10:17</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>76</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>09:01:57</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>77</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>08:46:31</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>92</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>09:01:57</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>10:29</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>88</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>08:46:31</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="D23" t="n">
         <v>104</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2378
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E98"/>
+  <dimension ref="A1:E117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:01:57</t>
+          <t>Última actualización: 10:19:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 93</t>
+          <t>Total filas: 112</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2648,21 +2648,21 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>09:01:57</t>
+          <t>10:19:13</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>10:19</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2678,16 +2678,16 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:24</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>09:01:57</t>
+          <t>10:19:13</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:25</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>102</v>
+        <v>6</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>10:19:13</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:34</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>118</v>
+        <v>15</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2753,16 +2753,16 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>10:54</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,23 +2773,498 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>25</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>31</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>32</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
           <t>09:01:57</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>10:54</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>113</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>36</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>09:01:57</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
         <is>
           <t>10:56</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
+      <c r="C103" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D98" t="n">
+      <c r="D103" t="n">
         <v>115</v>
       </c>
-      <c r="E98" t="inlineStr">
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>38</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>46</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>49</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>56</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>11:24</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>65</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>11:32</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>73</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>76</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>11:36</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>77</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>11:41</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>82</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>86</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>95</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>96</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>105</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>116</v>
+      </c>
+      <c r="E117" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2806,7 +3281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2819,14 +3294,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:01:57</t>
+          <t>Última actualización: 10:19:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -3352,6 +3827,81 @@
         <v>99</v>
       </c>
       <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>10:19</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>76</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>86</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3368,7 +3918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3381,14 +3931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:01:57</t>
+          <t>Última actualización: 10:19:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -3822,50 +4372,125 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>09:01:57</t>
+          <t>10:19:13</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10:29</t>
+          <t>10:22</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>88</v>
+        <v>3</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>10:29</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>88</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>104</v>
-      </c>
-      <c r="E23" t="inlineStr">
+      <c r="D24" t="n">
+        <v>11</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>24</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>11:41</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>82</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2379
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E117"/>
+  <dimension ref="A1:E128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:19:13</t>
+          <t>Última actualización: 11:02:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 112</t>
+          <t>Total filas: 123</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>10:19:13</t>
+          <t>11:02:50</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>11:05</t>
+          <t>11:02</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>10:19:13</t>
+          <t>11:02:50</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>49</v>
+        <v>2</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:19:13</t>
+          <t>11:02:50</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>11:15</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3028,16 +3028,16 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>11:24</t>
+          <t>11:05</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,21 +3048,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:19:13</t>
+          <t>11:02:50</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>11:32</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>73</v>
+        <v>6</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:19:13</t>
+          <t>11:02:50</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>11:35</t>
+          <t>11:15</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>76</v>
+        <v>13</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>10:19:13</t>
+          <t>11:02:50</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>11:36</t>
+          <t>11:24</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>77</v>
+        <v>22</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3128,16 +3128,16 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>11:41</t>
+          <t>11:32</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>10:19:13</t>
+          <t>11:02:50</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>11:34</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>86</v>
+        <v>32</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3178,16 +3178,16 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>11:54</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3203,16 +3203,16 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:36</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,21 +3223,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>10:19:13</t>
+          <t>11:02:50</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>11:41</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>105</v>
+        <v>39</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,23 +3248,298 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
+          <t>11:02:50</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>42</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
           <t>10:19:13</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr">
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>86</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>11:02:50</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>52</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>11:02:50</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>53</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>11:02:50</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>12:02</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>60</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>11:02:50</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>62</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>11:02:50</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
+      <c r="C123" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D117" t="n">
-        <v>116</v>
-      </c>
-      <c r="E117" t="inlineStr">
+      <c r="D123" t="n">
+        <v>73</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>11:02:50</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>12:24</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>82</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>11:02:50</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>12:31</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>89</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>11:02:50</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>92</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>11:02:50</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>94</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>11:02:50</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>12:43</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>101</v>
+      </c>
+      <c r="E128" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3281,7 +3556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3294,14 +3569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:19:13</t>
+          <t>Última actualización: 11:02:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -3645,7 +3920,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -3670,7 +3945,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -3860,12 +4135,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>10:19:13</t>
+          <t>11:02:50</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>11:35</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3874,7 +4149,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>76</v>
+        <v>2</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -3885,23 +4160,98 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>11:02:50</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>32</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>10:19:13</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>76</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>11:02:50</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>42</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>10:19:13</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>11:45</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="D31" t="n">
         <v>86</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3918,7 +4268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3931,14 +4281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:19:13</t>
+          <t>Última actualización: 11:02:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -4322,7 +4672,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>09:01:57</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -4332,22 +4682,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -4357,15 +4707,15 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
@@ -4489,6 +4839,31 @@
         <v>82</v>
       </c>
       <c r="E26" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>11:02:50</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>83</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2380
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E128"/>
+  <dimension ref="A1:E140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:02:50</t>
+          <t>Última actualización: 11:49:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 123</t>
+          <t>Total filas: 135</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3298,7 +3298,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>11:02:50</t>
+          <t>11:49:24</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>52</v>
+        <v>5</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>11:02:50</t>
+          <t>11:49:24</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3337,7 +3337,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>53</v>
+        <v>6</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>11:02:50</t>
+          <t>11:49:24</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3387,7 +3387,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>62</v>
+        <v>15</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>11:02:50</t>
+          <t>11:49:24</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:07</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>73</v>
+        <v>18</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>11:02:50</t>
+          <t>11:49:24</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:11</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>82</v>
+        <v>22</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>11:02:50</t>
+          <t>11:49:24</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>89</v>
+        <v>26</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>11:02:50</t>
+          <t>11:49:24</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>92</v>
+        <v>35</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>11:02:50</t>
+          <t>11:49:24</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>94</v>
+        <v>42</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,23 +3523,323 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
+          <t>11:49:24</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>45</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
           <t>11:02:50</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr">
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>94</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>11:02:50</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
         <is>
           <t>12:43</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr">
+      <c r="C130" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D128" t="n">
+      <c r="D130" t="n">
         <v>101</v>
       </c>
-      <c r="E128" t="inlineStr">
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>11:49:24</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>55</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>11:49:24</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>57</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>11:49:24</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>66</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>11:49:24</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>75</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>11:49:24</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>86</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>11:49:24</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>92</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>11:49:24</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>95</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>11:49:24</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>102</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>11:49:24</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>13:44</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>115</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>11:49:24</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>118</v>
+      </c>
+      <c r="E140" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3556,7 +3856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3569,14 +3869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:02:50</t>
+          <t>Última actualización: 11:49:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -3870,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -3895,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4252,6 +4552,56 @@
         <v>86</v>
       </c>
       <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>11:49:24</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>66</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>11:49:24</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>102</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4268,7 +4618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4281,14 +4631,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:02:50</t>
+          <t>Última actualización: 11:49:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -4672,7 +5022,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -4682,22 +5032,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>09:01:57</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -4707,15 +5057,15 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
@@ -4864,6 +5214,56 @@
         <v>83</v>
       </c>
       <c r="E27" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>11:49:24</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>65</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>11:49:24</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>94</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2381
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:49:24</t>
+          <t>Última actualización: 12:19:33</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>06:23:26</t>
+          <t>07:50:06</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>88</v>
+        <v>1</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:50:06</t>
+          <t>06:23:26</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>1</v>
+        <v>88</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:49:24</t>
+          <t>Última actualización: 12:19:33</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4618,7 +4618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4631,14 +4631,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:49:24</t>
+          <t>Última actualización: 12:19:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -5022,7 +5022,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>09:01:57</t>
+          <t>08:46:31</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -5032,22 +5032,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>08:46:31</t>
+          <t>09:01:57</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -5057,15 +5057,15 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
@@ -5247,23 +5247,48 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>12:19:32</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>12:59</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>40</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>11:49:24</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>13:23</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D30" t="n">
         <v>94</v>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2382
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:19:33</t>
+          <t>Última actualización: 12:49:26</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:19:33</t>
+          <t>Última actualización: 12:49:26</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4631,7 +4631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:19:33</t>
+          <t>Última actualización: 12:49:26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2383
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:49:26</t>
+          <t>Última actualización: 13:17:37</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:49:26</t>
+          <t>Última actualización: 13:17:37</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4618,7 +4618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4631,14 +4631,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:49:26</t>
+          <t>Última actualización: 13:17:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -5291,6 +5291,31 @@
       <c r="E30" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>13:17:37</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>14:36</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>79</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2384
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:17:37</t>
+          <t>Última actualización: 13:56:50</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:17:37</t>
+          <t>Última actualización: 13:56:50</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4631,7 +4631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:17:37</t>
+          <t>Última actualización: 13:56:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2385
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:56:50</t>
+          <t>Última actualización: 14:24:40</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:56:50</t>
+          <t>Última actualización: 14:24:40</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4631,7 +4631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:56:50</t>
+          <t>Última actualización: 14:24:40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2386
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:24:40</t>
+          <t>Última actualización: 14:54:04</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:24:40</t>
+          <t>Última actualización: 14:54:04</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4631,7 +4631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:24:40</t>
+          <t>Última actualización: 14:54:04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2387
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:54:04</t>
+          <t>Última actualización: 15:27:07</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:54:04</t>
+          <t>Última actualización: 15:27:07</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4631,7 +4631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:54:04</t>
+          <t>Última actualización: 15:27:07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2388
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:27:07</t>
+          <t>Última actualización: 16:09:46</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:27:07</t>
+          <t>Última actualización: 16:09:46</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4631,7 +4631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:27:07</t>
+          <t>Última actualización: 16:09:46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2389
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:09:46</t>
+          <t>Última actualización: 16:47:37</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:09:46</t>
+          <t>Última actualización: 16:47:37</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4631,7 +4631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:09:46</t>
+          <t>Última actualización: 16:47:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2390
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:47:37</t>
+          <t>Última actualización: 17:02:51</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:47:37</t>
+          <t>Última actualización: 17:02:51</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4631,7 +4631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:47:37</t>
+          <t>Última actualización: 17:02:51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2391
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:02:51</t>
+          <t>Última actualización: 17:48:18</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:02:51</t>
+          <t>Última actualización: 17:48:18</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4631,7 +4631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:02:51</t>
+          <t>Última actualización: 17:48:18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2392
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:48:18</t>
+          <t>Última actualización: 18:17:12</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:48:18</t>
+          <t>Última actualización: 18:17:12</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4631,7 +4631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:48:18</t>
+          <t>Última actualización: 18:17:12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2393
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:17:12</t>
+          <t>Última actualización: 18:49:28</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:17:12</t>
+          <t>Última actualización: 18:49:28</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4631,7 +4631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:17:12</t>
+          <t>Última actualización: 18:49:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2394
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:49:28</t>
+          <t>Última actualización: 19:14:20</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:49:28</t>
+          <t>Última actualización: 19:14:20</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4631,7 +4631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:49:28</t>
+          <t>Última actualización: 19:14:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2395
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:14:20</t>
+          <t>Última actualización: 19:52:33</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:14:20</t>
+          <t>Última actualización: 19:52:33</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4631,7 +4631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:14:20</t>
+          <t>Última actualización: 19:52:33</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2396
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:52:33</t>
+          <t>Última actualización: 20:22:21</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:52:33</t>
+          <t>Última actualización: 20:22:21</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4631,7 +4631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:52:33</t>
+          <t>Última actualización: 20:22:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2397
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:22:21</t>
+          <t>Última actualización: 20:55:13</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:22:21</t>
+          <t>Última actualización: 20:55:13</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4631,7 +4631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:22:21</t>
+          <t>Última actualización: 20:55:13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2398
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-11.xlsx
+++ b/data/horarios-141-2026-04-11.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:55:13</t>
+          <t>Última actualización: 22:20:36</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3869,7 +3869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:55:13</t>
+          <t>Última actualización: 22:20:36</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4631,7 +4631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:55:13</t>
+          <t>Última actualización: 22:20:36</t>
         </is>
       </c>
     </row>

</xml_diff>